<commit_message>
Ajout des slides, module et generateur FX2 dans le repo
</commit_message>
<xml_diff>
--- a/_objectifs/Objectifs_et_couverture.xlsx
+++ b/_objectifs/Objectifs_et_couverture.xlsx
@@ -16,8 +16,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Modules'!$A$4:$K$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Exercices'!$A$4:$F$82</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Objectifs par module'!$A$4:$E$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Exercices'!$A$4:$F$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Objectifs par module'!$A$4:$E$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1912,11 +1912,11 @@
       </c>
       <c r="D18" s="17" t="inlineStr">
         <is>
-          <t>10, 11</t>
+          <t>09, 10, 11</t>
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F18" s="17" t="n">
         <v>0</v>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="I18" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J18" s="15" t="inlineStr">
         <is>
@@ -2226,7 +2226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F92"/>
+  <dimension ref="A1:F93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4408,12 +4408,12 @@
       </c>
       <c r="C71" s="28" t="inlineStr">
         <is>
-          <t>Une calculatrice, en MVC et FXML</t>
-        </is>
-      </c>
-      <c r="D71" s="30" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>Lier plutôt qu'écouter : bindings</t>
+        </is>
+      </c>
+      <c r="D71" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
         </is>
       </c>
       <c r="E71" s="26" t="inlineStr">
@@ -4440,12 +4440,12 @@
       </c>
       <c r="C72" s="28" t="inlineStr">
         <is>
-          <t>Le guichet : threads et Platform.runLater</t>
-        </is>
-      </c>
-      <c r="D72" s="31" t="inlineStr">
-        <is>
-          <t>Won't</t>
+          <t>Une calculatrice, en MVC et FXML</t>
+        </is>
+      </c>
+      <c r="D72" s="30" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="E72" s="26" t="inlineStr">
@@ -4453,41 +4453,41 @@
           <t>A.5</t>
         </is>
       </c>
-      <c r="F72" s="32" t="inlineStr">
-        <is>
-          <t>hors examen</t>
+      <c r="F72" s="26" t="inlineStr">
+        <is>
+          <t>livré</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="26" t="inlineStr">
         <is>
-          <t>FIC</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="B73" s="27" t="inlineStr">
         <is>
-          <t>FIC.1</t>
+          <t>FX.10</t>
         </is>
       </c>
       <c r="C73" s="28" t="inlineStr">
         <is>
-          <t>Trois classes qui se connaissent</t>
-        </is>
-      </c>
-      <c r="D73" s="30" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>Le guichet : threads et Platform.runLater</t>
+        </is>
+      </c>
+      <c r="D73" s="31" t="inlineStr">
+        <is>
+          <t>Won't</t>
         </is>
       </c>
       <c r="E73" s="26" t="inlineStr">
         <is>
-          <t>A.1</t>
-        </is>
-      </c>
-      <c r="F73" s="26" t="inlineStr">
-        <is>
-          <t>livré</t>
+          <t>A.5</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>hors examen</t>
         </is>
       </c>
     </row>
@@ -4499,22 +4499,22 @@
       </c>
       <c r="B74" s="27" t="inlineStr">
         <is>
-          <t>FIC.2</t>
+          <t>FIC.1</t>
         </is>
       </c>
       <c r="C74" s="28" t="inlineStr">
         <is>
-          <t>Enregistrer des objets</t>
-        </is>
-      </c>
-      <c r="D74" s="29" t="inlineStr">
-        <is>
-          <t>Must</t>
+          <t>Trois classes qui se connaissent</t>
+        </is>
+      </c>
+      <c r="D74" s="30" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="E74" s="26" t="inlineStr">
         <is>
-          <t>A.5</t>
+          <t>A.1</t>
         </is>
       </c>
       <c r="F74" s="26" t="inlineStr">
@@ -4531,17 +4531,17 @@
       </c>
       <c r="B75" s="27" t="inlineStr">
         <is>
-          <t>FIC.3</t>
+          <t>FIC.2</t>
         </is>
       </c>
       <c r="C75" s="28" t="inlineStr">
         <is>
-          <t>Enregistrer du texte</t>
-        </is>
-      </c>
-      <c r="D75" s="30" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>Enregistrer des objets</t>
+        </is>
+      </c>
+      <c r="D75" s="29" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="E75" s="26" t="inlineStr">
@@ -4558,54 +4558,54 @@
     <row r="76">
       <c r="A76" s="26" t="inlineStr">
         <is>
-          <t>REC</t>
+          <t>FIC</t>
         </is>
       </c>
       <c r="B76" s="27" t="inlineStr">
         <is>
-          <t>REC.*</t>
+          <t>FIC.3</t>
         </is>
       </c>
       <c r="C76" s="28" t="inlineStr">
         <is>
-          <t>Récapitulatifs — format et place à décider</t>
-        </is>
-      </c>
-      <c r="D76" s="31" t="inlineStr">
-        <is>
-          <t>Could</t>
+          <t>Enregistrer du texte</t>
+        </is>
+      </c>
+      <c r="D76" s="30" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="E76" s="26" t="inlineStr">
         <is>
-          <t>A.1</t>
-        </is>
-      </c>
-      <c r="F76" s="32" t="inlineStr">
-        <is>
-          <t>en attente</t>
+          <t>A.5</t>
+        </is>
+      </c>
+      <c r="F76" s="26" t="inlineStr">
+        <is>
+          <t>livré</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="26" t="inlineStr">
         <is>
-          <t>GAM</t>
+          <t>REC</t>
         </is>
       </c>
       <c r="B77" s="27" t="inlineStr">
         <is>
-          <t>G.1–G.9</t>
+          <t>REC.*</t>
         </is>
       </c>
       <c r="C77" s="28" t="inlineStr">
         <is>
-          <t>Le modèle : joueur, partie, énumérations, record</t>
-        </is>
-      </c>
-      <c r="D77" s="30" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>Récapitulatifs — format et place à décider</t>
+        </is>
+      </c>
+      <c r="D77" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
         </is>
       </c>
       <c r="E77" s="26" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="F77" s="32" t="inlineStr">
         <is>
-          <t>corrigé</t>
+          <t>en attente</t>
         </is>
       </c>
     </row>
@@ -4627,12 +4627,12 @@
       </c>
       <c r="B78" s="27" t="inlineStr">
         <is>
-          <t>G.10–G.13</t>
+          <t>G.1–G.9</t>
         </is>
       </c>
       <c r="C78" s="28" t="inlineStr">
         <is>
-          <t>Classe abstraite et patron Observateur</t>
+          <t>Le modèle : joueur, partie, énumérations, record</t>
         </is>
       </c>
       <c r="D78" s="30" t="inlineStr">
@@ -4642,7 +4642,7 @@
       </c>
       <c r="E78" s="26" t="inlineStr">
         <is>
-          <t>A.4</t>
+          <t>A.1</t>
         </is>
       </c>
       <c r="F78" s="32" t="inlineStr">
@@ -4659,22 +4659,22 @@
       </c>
       <c r="B79" s="27" t="inlineStr">
         <is>
-          <t>G.14–G.20</t>
+          <t>G.10–G.13</t>
         </is>
       </c>
       <c r="C79" s="28" t="inlineStr">
         <is>
-          <t>Interface Jeu, fabrique, Nim, stratégies</t>
-        </is>
-      </c>
-      <c r="D79" s="29" t="inlineStr">
-        <is>
-          <t>Must</t>
+          <t>Classe abstraite et patron Observateur</t>
+        </is>
+      </c>
+      <c r="D79" s="30" t="inlineStr">
+        <is>
+          <t>Should</t>
         </is>
       </c>
       <c r="E79" s="26" t="inlineStr">
         <is>
-          <t>C.1</t>
+          <t>A.4</t>
         </is>
       </c>
       <c r="F79" s="32" t="inlineStr">
@@ -4691,22 +4691,22 @@
       </c>
       <c r="B80" s="27" t="inlineStr">
         <is>
-          <t>G.21–G.27</t>
+          <t>G.14–G.20</t>
         </is>
       </c>
       <c r="C80" s="28" t="inlineStr">
         <is>
-          <t>Le jeu de bataille</t>
-        </is>
-      </c>
-      <c r="D80" s="31" t="inlineStr">
-        <is>
-          <t>Could</t>
+          <t>Interface Jeu, fabrique, Nim, stratégies</t>
+        </is>
+      </c>
+      <c r="D80" s="29" t="inlineStr">
+        <is>
+          <t>Must</t>
         </is>
       </c>
       <c r="E80" s="26" t="inlineStr">
         <is>
-          <t>A.3</t>
+          <t>C.1</t>
         </is>
       </c>
       <c r="F80" s="32" t="inlineStr">
@@ -4723,22 +4723,22 @@
       </c>
       <c r="B81" s="27" t="inlineStr">
         <is>
-          <t>G.21</t>
+          <t>G.21–G.27</t>
         </is>
       </c>
       <c r="C81" s="28" t="inlineStr">
         <is>
-          <t>Un jeu qui se joue seul</t>
-        </is>
-      </c>
-      <c r="D81" s="30" t="inlineStr">
-        <is>
-          <t>Should</t>
+          <t>Le jeu de bataille</t>
+        </is>
+      </c>
+      <c r="D81" s="31" t="inlineStr">
+        <is>
+          <t>Could</t>
         </is>
       </c>
       <c r="E81" s="26" t="inlineStr">
         <is>
-          <t>C.1</t>
+          <t>A.3</t>
         </is>
       </c>
       <c r="F81" s="32" t="inlineStr">
@@ -4755,107 +4755,139 @@
       </c>
       <c r="B82" s="27" t="inlineStr">
         <is>
+          <t>G.21</t>
+        </is>
+      </c>
+      <c r="C82" s="28" t="inlineStr">
+        <is>
+          <t>Un jeu qui se joue seul</t>
+        </is>
+      </c>
+      <c r="D82" s="30" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="E82" s="26" t="inlineStr">
+        <is>
+          <t>C.1</t>
+        </is>
+      </c>
+      <c r="F82" s="32" t="inlineStr">
+        <is>
+          <t>corrigé</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="26" t="inlineStr">
+        <is>
+          <t>GAM</t>
+        </is>
+      </c>
+      <c r="B83" s="27" t="inlineStr">
+        <is>
           <t>G.22</t>
         </is>
       </c>
-      <c r="C82" s="28" t="inlineStr">
+      <c r="C83" s="28" t="inlineStr">
         <is>
           <t>Un jeu qui ouvre une fenêtre</t>
         </is>
       </c>
-      <c r="D82" s="31" t="inlineStr">
+      <c r="D83" s="31" t="inlineStr">
         <is>
           <t>Could</t>
         </is>
       </c>
-      <c r="E82" s="26" t="inlineStr">
+      <c r="E83" s="26" t="inlineStr">
         <is>
           <t>A.5</t>
         </is>
       </c>
-      <c r="F82" s="32" t="inlineStr">
+      <c r="F83" s="32" t="inlineStr">
         <is>
           <t>corrigé</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="10" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>Combien d'exercices selon le scénario</t>
         </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="33" t="inlineStr">
-        <is>
-          <t>Must seuls</t>
-        </is>
-      </c>
-      <c r="B86" s="18">
-        <f>COUNTIF($D$5:$D$82,"Must")</f>
-        <v/>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="33" t="inlineStr">
         <is>
-          <t>Must + Should</t>
+          <t>Must seuls</t>
         </is>
       </c>
       <c r="B87" s="18">
-        <f>COUNTIF($D$5:$D$82,"Must")+COUNTIF($D$5:$D$82,"Should")</f>
+        <f>COUNTIF($D$5:$D$83,"Must")</f>
         <v/>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="33" t="inlineStr">
         <is>
-          <t>Tout sauf les Won't</t>
+          <t>Must + Should</t>
         </is>
       </c>
       <c r="B88" s="18">
-        <f>COUNTA($D$5:$D$82)-COUNTIF($D$5:$D$82,"Won't")</f>
+        <f>COUNTIF($D$5:$D$83,"Must")+COUNTIF($D$5:$D$83,"Should")</f>
         <v/>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="33" t="inlineStr">
         <is>
-          <t>Déjà livrés</t>
+          <t>Tout sauf les Won't</t>
         </is>
       </c>
       <c r="B89" s="18">
-        <f>COUNTIF($F$5:$F$82,"livré")</f>
+        <f>COUNTA($D$5:$D$83)-COUNTIF($D$5:$D$83,"Won't")</f>
         <v/>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="33" t="inlineStr">
         <is>
+          <t>Déjà livrés</t>
+        </is>
+      </c>
+      <c r="B90" s="18">
+        <f>COUNTIF($F$5:$F$83,"livré")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="33" t="inlineStr">
+        <is>
           <t>Restant à écrire</t>
         </is>
       </c>
-      <c r="B90" s="18">
-        <f>COUNTIF($F$5:$F$82,"à écrire")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="25" t="inlineStr">
+      <c r="B91" s="18">
+        <f>COUNTIF($F$5:$F$83,"à écrire")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="25" t="inlineStr">
         <is>
           <t>REC compte pour une seule ligne : son format n'est pas arrêté.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F82"/>
+  <autoFilter ref="A4:F83"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81 D82 D83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4869,7 +4901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E81"/>
+  <dimension ref="A1:E83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6617,7 +6649,7 @@
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>FX.1, FX.6</t>
+          <t>FX.1, FX.3</t>
         </is>
       </c>
     </row>
@@ -6644,7 +6676,7 @@
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>FX.2</t>
+          <t>FX.1, FX.2</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6703,7 @@
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>FX.3, FX.4</t>
+          <t>FX.4, FX.5</t>
         </is>
       </c>
     </row>
@@ -6725,7 +6757,7 @@
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>FX.6</t>
+          <t>FX.9</t>
         </is>
       </c>
     </row>
@@ -6752,61 +6784,61 @@
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>FX.7, FX.8</t>
+          <t>FX.9</t>
         </is>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="34" t="inlineStr">
         <is>
-          <t>FIC</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="B73" s="13" t="inlineStr">
         <is>
-          <t>FIC.a</t>
+          <t>FX.g</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>Modéliser un petit domaine à trois classes liées</t>
+          <t>Observer une propriété par un ChangeListener (facultatif)</t>
         </is>
       </c>
       <c r="D73" s="35" t="inlineStr">
         <is>
-          <t>A.1</t>
+          <t>A.5</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>FIC.1</t>
+          <t>FX.6, FX.7</t>
         </is>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="34" t="inlineStr">
         <is>
-          <t>FIC</t>
+          <t>FX</t>
         </is>
       </c>
       <c r="B74" s="13" t="inlineStr">
         <is>
-          <t>FIC.b</t>
+          <t>FX.h</t>
         </is>
       </c>
       <c r="C74" s="12" t="inlineStr">
         <is>
-          <t>Protéger une collection interne rendue par un accesseur</t>
+          <t>Lier des valeurs par un binding (facultatif)</t>
         </is>
       </c>
       <c r="D74" s="35" t="inlineStr">
         <is>
-          <t>C.1</t>
+          <t>A.5</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>FIC.1</t>
+          <t>FX.8</t>
         </is>
       </c>
     </row>
@@ -6818,22 +6850,22 @@
       </c>
       <c r="B75" s="13" t="inlineStr">
         <is>
-          <t>FIC.c</t>
+          <t>FIC.a</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>Sérialiser des objets et les relire</t>
+          <t>Modéliser un petit domaine à trois classes liées</t>
         </is>
       </c>
       <c r="D75" s="35" t="inlineStr">
         <is>
-          <t>A.5</t>
+          <t>A.1</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>FIC.2</t>
+          <t>FIC.1</t>
         </is>
       </c>
     </row>
@@ -6845,22 +6877,22 @@
       </c>
       <c r="B76" s="13" t="inlineStr">
         <is>
-          <t>FIC.d</t>
+          <t>FIC.b</t>
         </is>
       </c>
       <c r="C76" s="12" t="inlineStr">
         <is>
-          <t>Lire et écrire un fichier texte</t>
+          <t>Protéger une collection interne rendue par un accesseur</t>
         </is>
       </c>
       <c r="D76" s="35" t="inlineStr">
         <is>
-          <t>A.5</t>
+          <t>C.1</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>FIC.3</t>
+          <t>FIC.1</t>
         </is>
       </c>
     </row>
@@ -6872,94 +6904,148 @@
       </c>
       <c r="B77" s="13" t="inlineStr">
         <is>
+          <t>FIC.c</t>
+        </is>
+      </c>
+      <c r="C77" s="12" t="inlineStr">
+        <is>
+          <t>Sérialiser des objets et les relire</t>
+        </is>
+      </c>
+      <c r="D77" s="35" t="inlineStr">
+        <is>
+          <t>A.5</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>FIC.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="34" t="inlineStr">
+        <is>
+          <t>FIC</t>
+        </is>
+      </c>
+      <c r="B78" s="13" t="inlineStr">
+        <is>
+          <t>FIC.d</t>
+        </is>
+      </c>
+      <c r="C78" s="12" t="inlineStr">
+        <is>
+          <t>Lire et écrire un fichier texte</t>
+        </is>
+      </c>
+      <c r="D78" s="35" t="inlineStr">
+        <is>
+          <t>A.5</t>
+        </is>
+      </c>
+      <c r="E78" s="11" t="inlineStr">
+        <is>
+          <t>FIC.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="34" t="inlineStr">
+        <is>
+          <t>FIC</t>
+        </is>
+      </c>
+      <c r="B79" s="13" t="inlineStr">
+        <is>
           <t>FIC.e</t>
         </is>
       </c>
-      <c r="C77" s="12" t="inlineStr">
+      <c r="C79" s="12" t="inlineStr">
         <is>
           <t>Choisir un format en fonction de qui lira le fichier</t>
         </is>
       </c>
-      <c r="D77" s="35" t="inlineStr">
+      <c r="D79" s="35" t="inlineStr">
         <is>
           <t>C.1</t>
         </is>
       </c>
-      <c r="E77" s="11" t="inlineStr">
+      <c r="E79" s="11" t="inlineStr">
         <is>
           <t>FIC.3</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="36" t="inlineStr">
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="36" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B78" s="37" t="inlineStr">
+      <c r="B80" s="37" t="inlineStr">
         <is>
           <t>REC.a</t>
         </is>
       </c>
-      <c r="C78" s="38" t="inlineStr">
+      <c r="C80" s="38" t="inlineStr">
         <is>
           <t>Mobiliser plusieurs modules sur un même énoncé</t>
         </is>
       </c>
-      <c r="D78" s="35" t="inlineStr">
+      <c r="D80" s="35" t="inlineStr">
         <is>
           <t>A.1</t>
         </is>
       </c>
-      <c r="E78" s="39" t="inlineStr">
+      <c r="E80" s="39" t="inlineStr">
         <is>
           <t>à décider</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="22" customHeight="1">
-      <c r="A79" s="36" t="inlineStr">
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="36" t="inlineStr">
         <is>
           <t>REC</t>
         </is>
       </c>
-      <c r="B79" s="37" t="inlineStr">
+      <c r="B81" s="37" t="inlineStr">
         <is>
           <t>REC.b</t>
         </is>
       </c>
-      <c r="C79" s="38" t="inlineStr">
+      <c r="C81" s="38" t="inlineStr">
         <is>
           <t>Se préparer au format de l'examen</t>
         </is>
       </c>
-      <c r="D79" s="35" t="inlineStr">
+      <c r="D81" s="35" t="inlineStr">
         <is>
           <t>D.10</t>
         </is>
       </c>
-      <c r="E79" s="39" t="inlineStr">
+      <c r="E81" s="39" t="inlineStr">
         <is>
           <t>à décider</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="25" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="25" t="inlineStr">
         <is>
           <t>Fond rose : aucun exercice n'existe encore pour ce module. La couleur se déduit du disque, elle ne se décrète pas.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E79"/>
+  <autoFilter ref="A4:E81"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60 D61 D62 D63 D64 D65 D66 D67 D68 D69 D70 D71 D72 D73 D74 D75 D76 D77 D78 D79 D80 D81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A.1,A.2,A.3,A.4,A.5,A.6,B.1,B.2,B.3,C.1,C.2,D.1,D.2,D.3,D.4,D.5,D.6,D.7,D.8,D.9,D.10,D.11,D.12"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7126,67 +7212,67 @@
         </is>
       </c>
       <c r="C5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="D5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="E5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="F5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="G5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="H5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="I5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="J5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="K5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="L5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="M5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="N5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="O5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="P5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="Q5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="R5" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A5)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A5)</f>
         <v/>
       </c>
       <c r="S5" s="18">
@@ -7210,67 +7296,67 @@
         </is>
       </c>
       <c r="C6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="D6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="E6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="F6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="G6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="H6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="I6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="J6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="K6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="L6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="M6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="N6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="O6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="P6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="Q6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="R6" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A6)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A6)</f>
         <v/>
       </c>
       <c r="S6" s="18">
@@ -7294,67 +7380,67 @@
         </is>
       </c>
       <c r="C7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="D7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="E7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="F7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="G7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="H7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="I7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="J7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="K7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="L7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="M7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="N7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="O7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="P7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="Q7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="R7" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A7)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A7)</f>
         <v/>
       </c>
       <c r="S7" s="18">
@@ -7378,67 +7464,67 @@
         </is>
       </c>
       <c r="C8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="D8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="E8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="F8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="G8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="H8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="I8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="J8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="K8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="L8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="M8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="N8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="O8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="P8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="Q8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="R8" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A8)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A8)</f>
         <v/>
       </c>
       <c r="S8" s="18">
@@ -7462,67 +7548,67 @@
         </is>
       </c>
       <c r="C9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="D9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="E9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="F9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="G9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="H9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="I9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="J9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="K9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="L9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="M9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="N9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="O9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="P9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="Q9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="R9" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A9)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A9)</f>
         <v/>
       </c>
       <c r="S9" s="18">
@@ -7546,67 +7632,67 @@
         </is>
       </c>
       <c r="C10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="D10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="E10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="F10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="G10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="H10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="I10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="J10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="K10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="L10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="M10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="N10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="O10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="P10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="Q10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="R10" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A10)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A10)</f>
         <v/>
       </c>
       <c r="S10" s="18">
@@ -7630,67 +7716,67 @@
         </is>
       </c>
       <c r="C11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="D11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="E11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="F11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="G11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="H11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="I11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="J11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="K11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="L11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="M11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="N11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="O11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="P11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="Q11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="R11" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A11)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A11)</f>
         <v/>
       </c>
       <c r="S11" s="18">
@@ -7714,67 +7800,67 @@
         </is>
       </c>
       <c r="C12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="D12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="E12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="F12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="G12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="H12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="I12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="J12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="K12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="L12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="M12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="N12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="O12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="P12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="Q12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="R12" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A12)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A12)</f>
         <v/>
       </c>
       <c r="S12" s="18">
@@ -7798,67 +7884,67 @@
         </is>
       </c>
       <c r="C13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="D13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="E13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="F13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="G13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="H13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="I13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="J13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="K13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="L13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="M13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="N13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="O13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="P13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="Q13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="R13" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A13)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A13)</f>
         <v/>
       </c>
       <c r="S13" s="18">
@@ -7882,67 +7968,67 @@
         </is>
       </c>
       <c r="C14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="D14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="E14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="F14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="G14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="H14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="I14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="J14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="K14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="L14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="M14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="N14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="O14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="P14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="Q14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="R14" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A14)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A14)</f>
         <v/>
       </c>
       <c r="S14" s="18">
@@ -7966,67 +8052,67 @@
         </is>
       </c>
       <c r="C15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,C$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,C$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="D15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,D$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,D$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="E15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,E$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,E$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="F15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,F$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,F$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="G15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,G$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,G$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="H15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,H$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,H$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="I15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,I$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,I$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="J15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,J$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,J$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="K15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,K$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,K$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="L15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,L$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,L$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="M15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,M$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,M$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="N15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,N$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,N$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="O15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,O$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,O$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="P15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,P$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,P$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="Q15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,Q$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,Q$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="R15" s="42">
-        <f>COUNTIFS('Objectifs par module'!$A$5:$A$79,R$4,'Objectifs par module'!$D$5:$D$79,$A15)</f>
+        <f>COUNTIFS('Objectifs par module'!$A$5:$A$81,R$4,'Objectifs par module'!$D$5:$D$81,$A15)</f>
         <v/>
       </c>
       <c r="S15" s="18">
@@ -8081,7 +8167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -8279,7 +8365,7 @@
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="43" t="inlineStr">
         <is>
-          <t>Captures d'ecran sous Windows</t>
+          <t>JavaFX — FX.8 (bindings) et pom.xml</t>
         </is>
       </c>
       <c r="B12" s="45" t="inlineStr">
@@ -8290,12 +8376,30 @@
       <c r="C12" s="13" t="inlineStr"/>
       <c r="D12" s="12" t="inlineStr">
         <is>
+          <t>FX.8 et son corrige ont ete ecrits le 11/10 sans JavaFX disponible : ni compiles ni lances. La calculatrice est passee de e08 a e09 (package, FXML, fx:controller) : a relancer. Le pom designe desormais ClicApp (demos) et fx.e01 (exercices, solutions) pour javafx:run : a essayer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="43" t="inlineStr">
+        <is>
+          <t>Captures d'ecran sous Windows</t>
+        </is>
+      </c>
+      <c r="B13" s="45" t="inlineStr">
+        <is>
+          <t>a faire</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr"/>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
           <t>Les 23 captures du guide et du document Git viennent d'un macOS. Nice to have, voir le todo.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="46" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="46" t="inlineStr">
         <is>
           <t>Une verification qui trouve des defauts est une verification qui a servi. Les vingt-trois defauts listes ci-dessus etaient tous invisibles a la relecture du code.</t>
         </is>
@@ -8304,8 +8408,8 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A14:D14"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A15:D15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>